<commit_message>
update old new eval compare
</commit_message>
<xml_diff>
--- a/old_new_eval_compare/20251203_diffs_tagged_summary.xlsx
+++ b/old_new_eval_compare/20251203_diffs_tagged_summary.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>updated by algorithm</t>
+          <t>updated by ground truth</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>updated by ground truth</t>
+          <t>updated by algorithm</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -558,16 +558,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>updated by algorithm</t>
+          <t>updated by ground truth</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>true to false</t>
+          <t>false to true</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -578,16 +578,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>updated by ground truth</t>
+          <t>updated by algorithm</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>false to true</t>
+          <t>true to false</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -758,16 +758,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>updated by algorithm</t>
+          <t>updated by ground truth</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>true to false</t>
+          <t>false to true</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -783,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>false to true</t>
+          <t>true to false</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
@@ -798,7 +798,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>updated by ground truth</t>
+          <t>updated by algorithm</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -858,7 +858,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>updated by algorithm</t>
+          <t>updated by ground truth</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
@@ -883,11 +883,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>true to false</t>
+          <t>false to true</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -898,16 +898,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>updated by ground truth</t>
+          <t>updated by algorithm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>false to true</t>
+          <t>true to false</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>